<commit_message>
Automation Code Without AI Help Pt.2
</commit_message>
<xml_diff>
--- a/cypress/fixtures/excel/mf-item-class-milktea-test-data.xlsx
+++ b/cypress/fixtures/excel/mf-item-class-milktea-test-data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23145" windowHeight="9600" firstSheet="5" activeTab="9"/>
+    <workbookView windowWidth="23145" windowHeight="9600"/>
   </bookViews>
   <sheets>
     <sheet name="pageLoaditemClass" sheetId="50" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>description</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-001</t>
+    <t>POS-POSITIVE-TESTING-ITEMCLASS-001</t>
   </si>
   <si>
     <t>Should load the Item Classification master file page</t>
@@ -53,7 +53,7 @@
     <t>itemClassDesc</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-010</t>
+    <t>POS-POSITIVE-TESTING-ITEMCLASS-002</t>
   </si>
   <si>
     <t>should add a TEA item classification</t>
@@ -62,7 +62,7 @@
     <t>TEA</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-011</t>
+    <t>POS-POSITIVE-TESTING-ITEMCLASS-003</t>
   </si>
   <si>
     <t>should add a DL ADD ONS item classification</t>
@@ -71,7 +71,7 @@
     <t>DL ADD ONS</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-012</t>
+    <t>POS-POSITIVE-TESTING-ITEMCLASS-004</t>
   </si>
   <si>
     <t>should add a Beverage Ingredients item classification</t>
@@ -80,7 +80,7 @@
     <t>Beverage Ingredients</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-013</t>
+    <t>POS-POSITIVE-TESTING-ITEMCLASS-005</t>
   </si>
   <si>
     <t>should add a Beverages item classification</t>
@@ -89,7 +89,7 @@
     <t>Beverages</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-014</t>
+    <t>POS-POSITIVE-TESTING-ITEMCLASS-006</t>
   </si>
   <si>
     <t>should add a Drinkware Accessories item classification</t>
@@ -98,7 +98,7 @@
     <t>Drinkware Accessories</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-015</t>
+    <t>POS-POSITIVE-TESTING-ITEMCLASS-007</t>
   </si>
   <si>
     <t>should add a Finished Good item classification</t>
@@ -107,7 +107,7 @@
     <t>Finished Good</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-016</t>
+    <t>POS-POSITIVE-TESTING-ITEMCLASS-008</t>
   </si>
   <si>
     <t>should add a Oil-Based item classification</t>
@@ -116,7 +116,7 @@
     <t>Oil-Based</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-017</t>
+    <t>POS-POSITIVE-TESTING-ITEMCLASS-009</t>
   </si>
   <si>
     <t>should add a Packaging Materials item classification</t>
@@ -125,7 +125,7 @@
     <t>Packaging Materials</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-018</t>
+    <t>POS-POSITIVE-TESTING-ITEMCLASS-010</t>
   </si>
   <si>
     <t>should add a Raw Materials item classification</t>
@@ -140,7 +140,7 @@
     <t>updateitemClassDesc</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-019</t>
+    <t>POS-POSITIVE-TESTING-ITEMCLASS-011</t>
   </si>
   <si>
     <t>should edit the Alcoholic Beverages item classification</t>
@@ -152,7 +152,7 @@
     <t>Alcohol - Beverage</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-020</t>
+    <t>POS-POSITIVE-TESTING-ITEMCLASS-012</t>
   </si>
   <si>
     <t>should delete the Alcoholic Beverages item classification</t>
@@ -161,7 +161,7 @@
     <t>requireditemClassDescMessage</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-021</t>
+    <t>POS-NEGATIVE-TESTING-ITEMCLASS-001</t>
   </si>
   <si>
     <t>should validate required item classification description</t>
@@ -173,7 +173,7 @@
     <t>duplicateMessage</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-022</t>
+    <t>POS-NEGATIVE-TESTING-ITEMCLASS-002</t>
   </si>
   <si>
     <t>should not allow duplicate item classification description</t>
@@ -185,7 +185,7 @@
     <t>Item Classification already exists.</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-023</t>
+    <t>POS-NEGATIVE-TESTING-ITEMCLASS-003</t>
   </si>
   <si>
     <t>should not allow spaces-only item classification description</t>
@@ -197,7 +197,7 @@
     <t>maxLengthMessage</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-024</t>
+    <t>POS-NEGATIVE-TESTING-ITEMCLASS-004</t>
   </si>
   <si>
     <t>should not allow overly long item classification description</t>
@@ -215,7 +215,7 @@
     <t>seconditemClassDesc</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-025</t>
+    <t>POS-NEGATIVE-TESTING-ITEMCLASS-005</t>
   </si>
   <si>
     <t>should not allow editing a duplicate item classification description</t>
@@ -227,13 +227,13 @@
     <t>errorMessage</t>
   </si>
   <si>
-    <t>POS-ITEMCLASS-026</t>
+    <t>POS-NEGATIVE-TESTING-ITEMCLASS-006</t>
   </si>
   <si>
     <t>should not allow special characters as an item classification description</t>
   </si>
   <si>
-    <t>"© ™ ® à á â ñ ä ¢ £ ¥ € ! @ # $ ^ * _ + = &lt; &gt; ? ` ~ \" | \\ [ ] ; :</t>
+    <t>! @ # $ ^ * _ + = &lt; &gt; ? `</t>
   </si>
   <si>
     <t>ITEM CLASSIFICATION DESCRIPTION should only contain letters and numbers.</t>
@@ -1178,41 +1178,41 @@
     </dxf>
   </dxfs>
   <tableStyles count="7">
-    <tableStyle name="DAY 3 - Zreading ACTUAL DATA (B-style" pivot="0" count="4" xr9:uid="{F55BC6B7-39F2-4C1B-8DA1-E91DCE60FA94}">
+    <tableStyle name="DAY 3 - Zreading ACTUAL DATA (B-style" pivot="0" count="4" xr9:uid="{133BFDE7-7B7C-4854-B039-41945370A3B6}">
       <tableStyleElement type="wholeTable" dxfId="3"/>
       <tableStyleElement type="headerRow" dxfId="2"/>
       <tableStyleElement type="firstRowStripe" dxfId="1"/>
       <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
-    <tableStyle name="PAYMENT BY DINE TYPE REPORT-style" pivot="0" count="4" xr9:uid="{A7E787E8-2995-4C66-B449-C985E2EEACCB}">
+    <tableStyle name="PAYMENT BY DINE TYPE REPORT-style" pivot="0" count="4" xr9:uid="{91BC629B-8D5D-4940-989E-009819163EBC}">
       <tableStyleElement type="wholeTable" dxfId="7"/>
       <tableStyleElement type="headerRow" dxfId="6"/>
       <tableStyleElement type="firstRowStripe" dxfId="5"/>
       <tableStyleElement type="secondRowStripe" dxfId="4"/>
     </tableStyle>
-    <tableStyle name="PAYMENT BY DINE TYPE REPORT-style 2" pivot="0" count="2" xr9:uid="{95D183F6-41C6-4195-989F-3FF52655EF2F}">
+    <tableStyle name="PAYMENT BY DINE TYPE REPORT-style 2" pivot="0" count="2" xr9:uid="{87C7553B-ED08-433F-9A3A-D0FB4A480F25}">
       <tableStyleElement type="firstRowStripe" dxfId="9"/>
       <tableStyleElement type="secondRowStripe" dxfId="8"/>
     </tableStyle>
-    <tableStyle name="Sheet37-style" pivot="0" count="4" xr9:uid="{6266E33A-EE82-409B-9DF3-EA716CCFF22D}">
+    <tableStyle name="Sheet37-style" pivot="0" count="4" xr9:uid="{692310D9-ACE7-49F9-8F01-A59240B75112}">
       <tableStyleElement type="wholeTable" dxfId="13"/>
       <tableStyleElement type="headerRow" dxfId="12"/>
       <tableStyleElement type="firstRowStripe" dxfId="11"/>
       <tableStyleElement type="secondRowStripe" dxfId="10"/>
     </tableStyle>
-    <tableStyle name="DAY 2- Zreading ACTUAL DATA (TE-style" pivot="0" count="4" xr9:uid="{E142E728-BE72-4F13-9168-16780207EC80}">
+    <tableStyle name="DAY 2- Zreading ACTUAL DATA (TE-style" pivot="0" count="4" xr9:uid="{A538B72D-5735-4363-8994-369B86293573}">
       <tableStyleElement type="wholeTable" dxfId="17"/>
       <tableStyleElement type="headerRow" dxfId="16"/>
       <tableStyleElement type="firstRowStripe" dxfId="15"/>
       <tableStyleElement type="secondRowStripe" dxfId="14"/>
     </tableStyle>
-    <tableStyle name="DAY 2 - Zreading ACTUAL DATA (B-style" pivot="0" count="4" xr9:uid="{DB6A88AF-BEDE-44EC-BE71-D1043CDDB5FD}">
+    <tableStyle name="DAY 2 - Zreading ACTUAL DATA (B-style" pivot="0" count="4" xr9:uid="{88DF1F02-2AFC-4C64-A696-750D5AFC0514}">
       <tableStyleElement type="wholeTable" dxfId="21"/>
       <tableStyleElement type="headerRow" dxfId="20"/>
       <tableStyleElement type="firstRowStripe" dxfId="19"/>
       <tableStyleElement type="secondRowStripe" dxfId="18"/>
     </tableStyle>
-    <tableStyle name="Sheet38-style" pivot="0" count="4" xr9:uid="{203AA03E-DF19-44A5-876B-C61762FC5BE3}">
+    <tableStyle name="Sheet38-style" pivot="0" count="4" xr9:uid="{9A37DCE6-16A2-49B2-B400-BE1135E73AF5}">
       <tableStyleElement type="wholeTable" dxfId="25"/>
       <tableStyleElement type="headerRow" dxfId="24"/>
       <tableStyleElement type="firstRowStripe" dxfId="23"/>
@@ -1428,7 +1428,7 @@
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="12.75" outlineLevelRow="1" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="21.4285714285714" customWidth="1"/>
+    <col min="1" max="1" width="40.8571428571429" customWidth="1"/>
     <col min="2" max="2" width="62.8571428571429" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1460,7 +1460,7 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="12.75" outlineLevelRow="1" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="21.4285714285714" customWidth="1"/>
+    <col min="1" max="1" width="41.8571428571429" customWidth="1"/>
     <col min="2" max="2" width="49.1428571428571" customWidth="1"/>
     <col min="3" max="3" width="58.8571428571429" customWidth="1"/>
     <col min="4" max="4" width="31.8571428571429" customWidth="1"/>
@@ -1505,15 +1505,15 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultColWidth="12.6285714285714" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="3"/>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultColWidth="12.6285714285714" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="41.1428571428571" customWidth="1"/>
     <col min="2" max="2" width="54.2857142857143" customWidth="1"/>
-    <col min="3" max="4" width="50.8761904761905" customWidth="1"/>
+    <col min="3" max="3" width="50.8761904761905" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:4">
+    <row r="1" customHeight="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1523,9 +1523,8 @@
       <c r="C1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1"/>
-    </row>
-    <row r="2" customHeight="1" spans="1:4">
+    </row>
+    <row r="2" customHeight="1" spans="1:3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1535,9 +1534,8 @@
       <c r="C2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="1"/>
-    </row>
-    <row r="3" customHeight="1" spans="1:4">
+    </row>
+    <row r="3" customHeight="1" spans="1:3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1547,9 +1545,8 @@
       <c r="C3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="1"/>
-    </row>
-    <row r="4" customHeight="1" spans="1:4">
+    </row>
+    <row r="4" customHeight="1" spans="1:3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -1559,9 +1556,8 @@
       <c r="C4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="1"/>
-    </row>
-    <row r="5" customHeight="1" spans="1:4">
+    </row>
+    <row r="5" customHeight="1" spans="1:3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -1571,9 +1567,8 @@
       <c r="C5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="1"/>
-    </row>
-    <row r="6" customHeight="1" spans="1:4">
+    </row>
+    <row r="6" customHeight="1" spans="1:3">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -1583,9 +1578,8 @@
       <c r="C6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="1"/>
-    </row>
-    <row r="7" customHeight="1" spans="1:4">
+    </row>
+    <row r="7" customHeight="1" spans="1:3">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -1595,9 +1589,8 @@
       <c r="C7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="1"/>
-    </row>
-    <row r="8" customHeight="1" spans="1:4">
+    </row>
+    <row r="8" customHeight="1" spans="1:3">
       <c r="A8" t="s">
         <v>23</v>
       </c>
@@ -1607,9 +1600,8 @@
       <c r="C8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="1"/>
-    </row>
-    <row r="9" customHeight="1" spans="1:4">
+    </row>
+    <row r="9" customHeight="1" spans="1:3">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -1619,9 +1611,8 @@
       <c r="C9" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="1"/>
-    </row>
-    <row r="10" customHeight="1" spans="1:4">
+    </row>
+    <row r="10" customHeight="1" spans="1:3">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -1631,11 +1622,6 @@
       <c r="C10" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="1"/>
-    </row>
-    <row r="11" customHeight="1" spans="1:4">
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1649,7 +1635,7 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="12.75" outlineLevelRow="1" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="21.4285714285714" customWidth="1"/>
+    <col min="1" max="1" width="40.8571428571429" customWidth="1"/>
     <col min="2" max="2" width="49.1428571428571" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
     <col min="4" max="4" width="22.5714285714286" customWidth="1"/>
@@ -1692,16 +1678,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="12.75" outlineLevelRow="1" outlineLevelCol="3"/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="12.75" outlineLevelRow="1" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="21.4285714285714" customWidth="1"/>
+    <col min="1" max="1" width="40.8571428571429" customWidth="1"/>
     <col min="2" max="2" width="49.1428571428571" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="4" max="4" width="22.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1711,9 +1696,8 @@
       <c r="C1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1"/>
-    </row>
-    <row r="2" spans="1:4">
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>38</v>
       </c>
@@ -1723,7 +1707,6 @@
       <c r="C2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D2" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1734,16 +1717,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="12.75" outlineLevelRow="1" outlineLevelCol="3"/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="12.75" outlineLevelRow="1" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="21.4285714285714" customWidth="1"/>
+    <col min="1" max="1" width="41.8571428571429" customWidth="1"/>
     <col min="2" max="2" width="49.1428571428571" customWidth="1"/>
-    <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="4" max="4" width="22.5714285714286" customWidth="1"/>
+    <col min="3" max="3" width="69.4285714285714" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1753,9 +1735,8 @@
       <c r="C1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1"/>
-    </row>
-    <row r="2" spans="1:4">
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -1765,7 +1746,6 @@
       <c r="C2" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1779,7 +1759,7 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="12.75" outlineLevelRow="1" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="21.4285714285714" customWidth="1"/>
+    <col min="1" max="1" width="41.8571428571429" customWidth="1"/>
     <col min="2" max="2" width="49.1428571428571" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
     <col min="4" max="4" width="31.8571428571429" customWidth="1"/>
@@ -1825,10 +1805,10 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="12.75" outlineLevelRow="1" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="21.4285714285714" customWidth="1"/>
+    <col min="1" max="1" width="41.8571428571429" customWidth="1"/>
     <col min="2" max="2" width="49.1428571428571" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="4" max="4" width="31.8571428571429" customWidth="1"/>
+    <col min="4" max="4" width="69.4285714285714" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1871,7 +1851,7 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="12.75" outlineLevelRow="1" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="21.4285714285714" customWidth="1"/>
+    <col min="1" max="1" width="41.8571428571429" customWidth="1"/>
     <col min="2" max="2" width="49.1428571428571" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
     <col min="4" max="4" width="31.8571428571429" customWidth="1"/>
@@ -1917,7 +1897,7 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="12.75" outlineLevelRow="1" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="21.4285714285714" customWidth="1"/>
+    <col min="1" max="1" width="41.8571428571429" customWidth="1"/>
     <col min="2" max="2" width="49.1428571428571" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
     <col min="4" max="5" width="31.8571428571429" customWidth="1"/>

</xml_diff>